<commit_message>
Fix AI movement limits in challenge mode
</commit_message>
<xml_diff>
--- a/outputs/elite-ai-traits/elite-ai-traits.xlsx
+++ b/outputs/elite-ai-traits/elite-ai-traits.xlsx
@@ -8,16 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\codex_card\outputs\elite-ai-traits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5239B50-3D07-4541-8EDC-4299CECA7BB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2807328-696F-4215-B7A5-D81B9B16808E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="4965" windowWidth="20340" windowHeight="14745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14100" yWindow="2955" windowWidth="20340" windowHeight="14745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="初级词条" sheetId="1" r:id="rId1"/>
     <sheet name="中级词条" sheetId="2" r:id="rId2"/>
     <sheet name="高级词条" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -622,16 +635,16 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -907,24 +920,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.95" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="26" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
+      <c r="A2" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
     </row>
     <row r="4" spans="1:6" ht="24" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -986,13 +999,13 @@
       <c r="A7" s="11">
         <v>1003</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="25" t="s">
         <v>28</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="27" t="s">
+      <c r="D7" s="25" t="s">
         <v>29</v>
       </c>
       <c r="E7" s="17">
@@ -1004,13 +1017,13 @@
       <c r="A8" s="11">
         <v>1004</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="25" t="s">
         <v>30</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" s="25" t="s">
         <v>31</v>
       </c>
       <c r="E8" s="17">
@@ -1022,13 +1035,13 @@
       <c r="A9" s="11">
         <v>1005</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="25" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="D9" s="25" t="s">
         <v>34</v>
       </c>
       <c r="E9" s="17">
@@ -1040,13 +1053,13 @@
       <c r="A10" s="11">
         <v>1006</v>
       </c>
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="25" t="s">
         <v>33</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="25" t="s">
         <v>36</v>
       </c>
       <c r="E10" s="17">
@@ -1058,13 +1071,13 @@
       <c r="A11" s="11">
         <v>1007</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="25" t="s">
         <v>35</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="D11" s="25" t="s">
         <v>59</v>
       </c>
       <c r="E11" s="17">
@@ -1076,17 +1089,17 @@
       <c r="A12" s="11">
         <v>1008</v>
       </c>
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="25" t="s">
         <v>38</v>
       </c>
       <c r="C12" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="25" t="s">
         <v>37</v>
       </c>
       <c r="E12" s="17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="7"/>
     </row>
@@ -1094,13 +1107,13 @@
       <c r="A13" s="11">
         <v>1009</v>
       </c>
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="25" t="s">
         <v>39</v>
       </c>
       <c r="C13" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="27" t="s">
+      <c r="D13" s="25" t="s">
         <v>40</v>
       </c>
       <c r="E13" s="17">
@@ -1112,13 +1125,13 @@
       <c r="A14" s="11">
         <v>1010</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="25" t="s">
         <v>41</v>
       </c>
       <c r="C14" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="25" t="s">
         <v>42</v>
       </c>
       <c r="E14" s="17">
@@ -1130,13 +1143,13 @@
       <c r="A15" s="11">
         <v>1011</v>
       </c>
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="25" t="s">
         <v>67</v>
       </c>
       <c r="C15" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="27" t="s">
+      <c r="D15" s="25" t="s">
         <v>68</v>
       </c>
       <c r="E15" s="17">
@@ -1194,24 +1207,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.95" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
     </row>
     <row r="4" spans="1:6" ht="24" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -1255,7 +1268,7 @@
       <c r="A6" s="11">
         <v>2002</v>
       </c>
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="26" t="s">
         <v>52</v>
       </c>
       <c r="C6" s="20" t="s">
@@ -1273,13 +1286,13 @@
       <c r="A7" s="11">
         <v>2003</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="25" t="s">
         <v>54</v>
       </c>
       <c r="C7" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="27" t="s">
+      <c r="D7" s="25" t="s">
         <v>46</v>
       </c>
       <c r="E7" s="17">
@@ -1291,13 +1304,13 @@
       <c r="A8" s="11">
         <v>2004</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="25" t="s">
         <v>50</v>
       </c>
       <c r="C8" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" s="25" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="17">
@@ -1315,7 +1328,7 @@
       <c r="C9" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="D9" s="25" t="s">
         <v>49</v>
       </c>
       <c r="E9" s="17">
@@ -1327,13 +1340,13 @@
       <c r="A10" s="11">
         <v>2006</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="26" t="s">
         <v>53</v>
       </c>
       <c r="C10" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="25" t="s">
         <v>51</v>
       </c>
       <c r="E10" s="17">
@@ -1345,13 +1358,13 @@
       <c r="A11" s="11">
         <v>2007</v>
       </c>
-      <c r="B11" s="28" t="s">
+      <c r="B11" s="26" t="s">
         <v>55</v>
       </c>
       <c r="C11" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="D11" s="25" t="s">
         <v>56</v>
       </c>
       <c r="E11" s="17">
@@ -1369,7 +1382,7 @@
       <c r="C12" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="25" t="s">
         <v>58</v>
       </c>
       <c r="E12" s="17">
@@ -1427,24 +1440,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.95" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
     </row>
     <row r="4" spans="1:6" ht="24" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -1524,7 +1537,7 @@
       <c r="A8" s="11">
         <v>3004</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="25" t="s">
         <v>43</v>
       </c>
       <c r="C8" s="23" t="s">
@@ -1542,7 +1555,7 @@
       <c r="A9" s="11">
         <v>3005</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="25" t="s">
         <v>44</v>
       </c>
       <c r="C9" s="23" t="s">
@@ -1560,7 +1573,7 @@
       <c r="A10" s="11">
         <v>3006</v>
       </c>
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="25" t="s">
         <v>60</v>
       </c>
       <c r="C10" s="23" t="s">
@@ -1578,13 +1591,13 @@
       <c r="A11" s="11">
         <v>3007</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="25" t="s">
         <v>63</v>
       </c>
       <c r="C11" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="D11" s="25" t="s">
         <v>64</v>
       </c>
       <c r="E11" s="17">
@@ -1596,13 +1609,13 @@
       <c r="A12" s="11">
         <v>3008</v>
       </c>
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="25" t="s">
         <v>65</v>
       </c>
       <c r="C12" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="25" t="s">
         <v>66</v>
       </c>
       <c r="E12" s="17">

</xml_diff>